<commit_message>
Add tactical combat & mass specs; update assets
Add two Russian tactical specification Markdown files (Бой.Урон and МАССА,РОСТ,ПРИКРЫТИЕ,ПЛОЩАДЬ) replacing placeholder .txt files. Update several design/visual binary assets (XLSX, WEBP) and add new design resources under design/. These changes introduce combat and size-related rules and refresh related design materials.
</commit_message>
<xml_diff>
--- a/design/Справочные таблицы/Телосложение и Масса.xlsx
+++ b/design/Справочные таблицы/Телосложение и Масса.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="64">
   <si>
     <t>Название категории</t>
   </si>
@@ -137,27 +137,18 @@
     <t>+1 реакция</t>
   </si>
   <si>
-    <t>+7</t>
-  </si>
-  <si>
     <t>101-130</t>
   </si>
   <si>
     <t>Увесистый (6)</t>
   </si>
   <si>
-    <t>+5</t>
-  </si>
-  <si>
     <t>81-100</t>
   </si>
   <si>
     <t>Выше среднего (5)</t>
   </si>
   <si>
-    <t>+2</t>
-  </si>
-  <si>
     <t>66-80</t>
   </si>
   <si>
@@ -186,6 +177,36 @@
   </si>
   <si>
     <t>Менее 1</t>
+  </si>
+  <si>
+    <t>Площадь в клетках</t>
+  </si>
+  <si>
+    <t>4 (2х2)</t>
+  </si>
+  <si>
+    <t>4 или 6 (2х3)</t>
+  </si>
+  <si>
+    <t>2х1</t>
+  </si>
+  <si>
+    <t>Прикрытие в клетках</t>
+  </si>
+  <si>
+    <t>2х2 или 3х1</t>
+  </si>
+  <si>
+    <t>8 (2х4) или 9(3х3)</t>
+  </si>
+  <si>
+    <t>2х4 или 3х3</t>
+  </si>
+  <si>
+    <t>20 (4х5 или 5х4)</t>
+  </si>
+  <si>
+    <t>2х3 или 3х2</t>
   </si>
 </sst>
 </file>
@@ -260,7 +281,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -287,6 +308,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -590,16 +617,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="18.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.140625" customWidth="1"/>
     <col min="3" max="3" width="18.5703125" customWidth="1"/>
     <col min="4" max="5" width="18" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -618,8 +647,14 @@
       <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G1" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
@@ -638,8 +673,14 @@
       <c r="F2" s="3" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G2" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>7</v>
       </c>
@@ -658,8 +699,14 @@
       <c r="F3" s="5" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G3" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>10</v>
       </c>
@@ -678,8 +725,14 @@
       <c r="F4" s="3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>13</v>
       </c>
@@ -698,8 +751,14 @@
       <c r="F5" s="5" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="H5" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>16</v>
       </c>
@@ -718,8 +777,14 @@
       <c r="F6" s="3" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G6" s="3">
+        <v>1</v>
+      </c>
+      <c r="H6" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>18</v>
       </c>
@@ -738,8 +803,14 @@
       <c r="F7" s="5" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+      <c r="G7" s="5">
+        <v>1</v>
+      </c>
+      <c r="H7" s="5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -758,8 +829,14 @@
       <c r="F8" s="3" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="G8" s="3">
+        <v>1</v>
+      </c>
+      <c r="H8" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>24</v>
       </c>
@@ -777,6 +854,12 @@
       </c>
       <c r="F9" s="7" t="s">
         <v>25</v>
+      </c>
+      <c r="G9" s="7">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -874,16 +957,16 @@
       <c r="C5" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="10">
+        <v>7</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>40</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="3">
         <v>-1</v>
@@ -891,16 +974,16 @@
       <c r="C6" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>43</v>
+      <c r="D6" s="11">
+        <v>5</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B7" s="5">
         <v>-1</v>
@@ -908,11 +991,11 @@
       <c r="C7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="5" t="s">
-        <v>46</v>
+      <c r="D7" s="10">
+        <v>2</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -923,27 +1006,27 @@
         <v>0</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B9" s="5">
         <v>1</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E9" s="8">
         <v>45962</v>
@@ -951,16 +1034,16 @@
     </row>
     <row r="10" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B10" s="3">
         <v>1</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E10" s="9">
         <v>46296</v>
@@ -968,19 +1051,19 @@
     </row>
     <row r="11" spans="1:5" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B11" s="7">
         <v>1</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>